<commit_message>
feat: add --legacy-vat-code-box flag, file Q2 2026 under Q1's treatment
The GL-category-based Box logic (previous commit) is more correct, but
its biggest effect - reclassifying most flight margin from Box 3B to
1E - is a large swing Dima wants to file consistently with Q1 2026's
already-submitted treatment, not switch mid-year. Adds a flag to run
main_old.py with the category override disabled, falling back to the
vat_code-driven logic for every transaction (still includes the pandas
crash fix and the PAS-on-commission-leg fix - those are bugs, not a
methodology choice).

Regenerates Q2 2026 reports with this flag for filing. Q1'26 vs Q2'26
(both old/vat_code treatment):
  1A:  24,009 -> 19,260  (-19.8%)
  1E: 328,494 -> 416,345 (+26.7%)
  3B: 879,252 -> 771,182 (-12.3%)
ICP: 148 -> 168 customers, still ties to Box 3B in both quarters.
</commit_message>
<xml_diff>
--- a/output/VAT final report Q2'26.xlsx
+++ b/output/VAT final report Q2'26.xlsx
@@ -450,10 +450,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>22075</v>
+        <v>19260</v>
       </c>
       <c r="D2" t="n">
-        <v>4636</v>
+        <v>4045</v>
       </c>
     </row>
     <row r="3">
@@ -468,7 +468,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1087727</v>
+        <v>416345</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -486,10 +486,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>70681</v>
+        <v>771182</v>
       </c>
       <c r="D4" t="n">
-        <v>14843</v>
+        <v>161948</v>
       </c>
     </row>
     <row r="5">

</xml_diff>